<commit_message>
feat: add font-size setting rows + line-break note to template
</commit_message>
<xml_diff>
--- a/client_template.xlsx
+++ b/client_template.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,12 @@
       <i val="1"/>
       <color rgb="00808080"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002C5AA0"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -70,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -82,6 +88,7 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -485,7 +492,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>השם שמופיע בכותרת</t>
+          <t>השם שמופיע בכותרת — לירידת שורה, לחץ Alt+Enter בתוך התא</t>
         </is>
       </c>
     </row>
@@ -870,6 +877,182 @@
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>— גדלי פונטים (ריק = ברירת מחדל אוטומטית) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>גודל_שם_בניין</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>פיקסלים (למשל 40) — ריק = גודל אוטומטי לפי המסך</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>גודל_שעון</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>פיקסלים — ריק = אוטומטי</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>גודל_תאריך_עברי</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>פיקסלים — ריק = אוטומטי</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>גודל_תאריך_לועזי</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>פיקסלים — ריק = אוטומטי</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>גודל_כותרת_כרטיס</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>כותרות כרטיסים (הודעות/זמנים/שבת) — פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>גודל_כותרת_הודעה</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>כותרת כל הודעה בודדת — פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>גודל_טקסט_הודעה</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>טקסט כל הודעה בודדת — פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>גודל_תווית_זמן</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>תוויות בעמודת זמנים (למשל "נץ החמה") — פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>גודל_שעת_זמן</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>השעות עצמן בעמודת זמנים — פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>גודל_שעת_מזג_אוויר</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>גודל_טמפ_מזג_אוויר</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>גודל_פרטי_מזג_אוויר</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>רוח/גשם — פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>גודל_פוטר</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>פיקסלים</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add פריסת_תמונה setting row to template
</commit_message>
<xml_diff>
--- a/client_template.xlsx
+++ b/client_template.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1051,6 +1051,23 @@
       <c r="C42" s="3" t="inlineStr">
         <is>
           <t>פיקסלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>פריסת_תמונה</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>מותאם</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>מותאם = כל התמונה נכנסת (יתכן רווח בצדדים) | מלא = ממלא את המסגרת (יתכן חיתוך)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add weather mode settings to template
</commit_message>
<xml_diff>
--- a/client_template.xlsx
+++ b/client_template.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1068,6 +1068,40 @@
       <c r="C43" s="3" t="inlineStr">
         <is>
           <t>מותאם = כל התמונה נכנסת (יתכן רווח בצדדים) | מלא = ממלא את המסגרת (יתכן חיתוך)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>מצב_מזג_אוויר</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>שעות</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>שעות = תחזית שעתית | ימים = תחזית 5 ימים | גם_וגם = מתחלף אוטומטית</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>מרווח_מזג_אוויר</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>שניות בין מעבר שעות/ימים (רק במצב גם_וגם)</t>
         </is>
       </c>
     </row>

</xml_diff>